<commit_message>
feat: implement dashboard UI components for new sections like weiterempfehlung, teilnemende etc. and initialized new page, made the navbar and footer reusable in a single js file
</commit_message>
<xml_diff>
--- a/data/data.xlsx
+++ b/data/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamia\Documents\Quadriga\Dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{103B89AE-6E55-4203-9C46-BA4597A1EEAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6092C03-2932-4F8C-BC02-DBCC16E18F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aktive Kooperationen" sheetId="1" r:id="rId1"/>

</xml_diff>